<commit_message>
Update Glyph_Organizer2.xlsx with new Ravi, Nima, and Veynar storyline developments
- Enhanced Ravi and Nima entries with deeper emotional nuance and character development
- Added Veynar content establishing his rigid personality and conflict with Kaelen/Drossel
- Introduced nuance to player's choice: whether to trust Veynar's law enforcement or side with criminals
- Developed Veynar's motivation: hypervigilance stemming from unknown gaps in his own mind post-collapse

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Velinor-Unity/Documentation/Game_Planning/Glyph_Organizer2.xlsx
+++ b/Velinor-Unity/Documentation/Game_Planning/Glyph_Organizer2.xlsx
@@ -5,25 +5,25 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Velinor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\saoriverse-console\Velinor-Unity\Documentation\Game_Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36BDFC1F-875B-46DA-A677-A94D58DC5076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16350E4A-84CE-48B2-AE8C-DB6363326C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1EBE45AE-1D7A-4751-8346-F50CF97E851D}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{1EBE45AE-1D7A-4751-8346-F50CF97E851D}"/>
   </bookViews>
   <sheets>
     <sheet name="Glyph_Organizer" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Glyph_Organizer!$A$1:$I$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Glyph_Organizer!$A$1:$I$74</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="278">
   <si>
     <t>Category</t>
   </si>
@@ -145,9 +145,6 @@
     <t>Collapsing trade route.</t>
   </si>
   <si>
-    <t>Tovren teaches the player to mark unstable paths with chalk. Sovereignty is clarity ? boundaries drawn to protect travelers.</t>
-  </si>
-  <si>
     <t>Tala - Market Cook</t>
   </si>
   <si>
@@ -524,9 +521,6 @@
   </si>
   <si>
     <t>Glyph of Quiet Return</t>
-  </si>
-  <si>
-    <t>Helia tends to an unconscious survivor and doubts whether her presence matters. When the player quietly sits with them, the survivor briefly awakens, whispering for someone to stay. The glyph manifests as Helia realizes that presence â€” not action â€” is what brings people back to themselves.</t>
   </si>
   <si>
     <t>Glyph of Quiet Bloom</t>
@@ -909,6 +903,30 @@
     <t xml:space="preserve">Ressa is sharp as a tack and speaks like one too. She meets the player on her fifth day in Velhara's marketplace when a wall suddenly starts collapsing threatening to crush the player, who is distracted by a vagrant boy that tried to steal the filament from her jacket. She and others in the market yell out loudly to the player to move out of harm's way just in time. Ressa directs the player who is still looking for consistent, work, food and shelter to go see Malrik or Elenya. The player chooses Malrik first because he pays. 
 The glyph triggers on her second encounter with Ressa in which the player tells Ressa about her experiences with Malrik and Elenya and how different they are. The player also talks about how she felt when hearing about Ophina and appreciated Ressa for sparing her a similar fate. Appreciating the player's attittude Ressa tells the player why she has kind of a sixth sense about collapses. She reveals that when she first came to the marketplace she was there with a friend. A piece of building suddently fell on her friend and crushed his leg. He was unable to move around much. She still takes care of him though at her home. 
 The player is prompted to find the Glyph of Ceaseless Vigilance. On return she meets Ressa at her home and meets her friend as well Their relationship reminds the player about a boy that passed through the farm area and she befriended. He only could stay for a week and she never saw him again. </t>
+  </si>
+  <si>
+    <t>Nima</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Nima - Community Leader</t>
+  </si>
+  <si>
+    <t>Market outskirts</t>
+  </si>
+  <si>
+    <t>After the player returns from the triglyph chamber and reveals how the marketplace quietly supported Nima, Ophina, and Ravi, Nima is overwhelmed by guilt. Once a central pillar of community life, she now feels undeserving of belonging after shutting everyone out in her grief. The codex updates, directing the player to seek the Glyph of Quiet Return.
+Even after the player recovers and brings it to her, Nima remains convinced she has forfeited her place. Nearby, a distraught stranger refuses comfort from anyone in the crowd, yet keeps glancing toward Nima. Recognizing the same hollow ache she carried for a year, Nima instinctively sits beside them in silence. The stranger finally speaks, confiding their loss. In that quiet exchange, Nima understands that her grief does not disqualify her mission — it deepens it. Watching her, the player senses their own path toward belonging may be unfolding as well.</t>
+  </si>
+  <si>
+    <t>Ravi - Market Watchman</t>
+  </si>
+  <si>
+    <t>Post‑triglyph, Ravi admits he trusts too quickly to keep despair at bay. Veynar’s rigid vigilance unsettles him: Veynar sees danger everywhere, while Ravi sees nuance. The codex pulses, directing the player to seek the Glyph of Marked Boundaries.
+Following the signal, the player finds Veynar sealing off an active path and dismissing Ravi’s open‑trail markers as fatal softness. “Boundaries are the only thing that keep grief from repeating,” he warns. Between their opposing markers, the player activates the glyph pedestal.
+Returning the glyph, the player speaks to Ravi with firsthand experience of Veynar’s stance. Ravi realizes blind trust invites ruin, yet Veynar’s walls kill living connection. Grounded by the player’s steadiness, he resolves to choose trust deliberately rather than collapse into it. The glyph reflects the player’s own journey: sovereignty is not isolation, but choosing how and when to let others in.  The player leaves with a question: should they trust Veynar’s judgment, or be wary of what he is trying so hard to keep others away from?</t>
   </si>
 </sst>
 </file>
@@ -1413,7 +1431,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1442,6 +1460,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1849,7 +1887,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>5</v>
@@ -1858,7 +1896,7 @@
         <v>6</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -1872,566 +1910,568 @@
         <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="I2" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2">
+        <v>67</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="2">
-        <v>29</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>100</v>
-      </c>
       <c r="I4" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>180</v>
+        <v>97</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="10">
+        <v>35</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2">
+        <v>30</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2">
-        <v>30</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="2">
-        <v>68</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>195</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>58</v>
+        <v>257</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>193</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
-        <v>59</v>
+        <v>194</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>60</v>
+        <v>195</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>84</v>
+        <v>253</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>57</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>186</v>
+        <v>83</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>187</v>
+        <v>84</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>188</v>
+        <v>85</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="B11" s="2">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>164</v>
+        <v>185</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
       <c r="I11" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="2">
+        <v>52</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="2">
-        <v>73</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>167</v>
+        <v>224</v>
       </c>
       <c r="I12" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2">
+        <v>42</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="2">
-        <v>8</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
-        <v>46</v>
+        <v>148</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>47</v>
+        <v>225</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="165" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B14" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>145</v>
+        <v>234</v>
       </c>
       <c r="F14" s="2"/>
-      <c r="G14" s="2" t="s">
-        <v>146</v>
+      <c r="G14" s="1" t="s">
+        <v>236</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>147</v>
+        <v>237</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="180" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="2">
-        <v>50</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B15" s="2"/>
       <c r="C15" s="3" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>265</v>
+        <v>232</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>25</v>
+        <v>235</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
-        <v>26</v>
+        <v>240</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>27</v>
+        <v>241</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="210" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2">
         <v>28</v>
       </c>
+      <c r="B16" s="2"/>
       <c r="C16" s="3" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>218</v>
-      </c>
+        <v>233</v>
+      </c>
+      <c r="F16" s="2"/>
       <c r="G16" s="2" t="s">
-        <v>193</v>
+        <v>238</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>194</v>
+        <v>239</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="2">
-        <v>66</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B18" s="2">
-        <v>56</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" s="13" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="10">
+        <v>38</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" s="17" customFormat="1" ht="165" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="14">
+        <v>73</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14" t="s">
+        <v>274</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>275</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>266</v>
+        <v>247</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>177</v>
+        <v>44</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2" t="s">
-        <v>178</v>
+        <v>45</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>179</v>
+        <v>46</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B20" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>87</v>
+        <v>247</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2" t="s">
-        <v>88</v>
+        <v>145</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>89</v>
+        <v>146</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2" t="s">
-        <v>93</v>
+        <v>26</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>94</v>
+        <v>27</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="B22" s="2">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F22" s="2"/>
+        <v>190</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>216</v>
+      </c>
       <c r="G22" s="2" t="s">
-        <v>124</v>
+        <v>191</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>125</v>
+        <v>192</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -2439,1444 +2479,1439 @@
         <v>7</v>
       </c>
       <c r="B23" s="2">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>126</v>
+        <v>248</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" s="2">
+        <v>56</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="2">
-        <v>58</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>134</v>
+        <v>172</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2" t="s">
-        <v>135</v>
+        <v>173</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>136</v>
+        <v>174</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B25" s="2">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>152</v>
+        <v>106</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>107</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B26" s="2">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F26" s="2"/>
+        <v>197</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>215</v>
+      </c>
       <c r="G26" s="2" t="s">
-        <v>23</v>
+        <v>202</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>24</v>
+        <v>203</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="B27" s="2">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>12</v>
+        <v>175</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2" t="s">
-        <v>13</v>
+        <v>176</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>14</v>
+        <v>177</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="165" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B28" s="2">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F28" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>216</v>
+      </c>
       <c r="G28" s="2" t="s">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>19</v>
+        <v>217</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B29" s="2">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2" t="s">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>51</v>
+        <v>88</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="B30" s="2">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>52</v>
+        <v>249</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2" t="s">
-        <v>53</v>
+        <v>92</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>54</v>
+        <v>93</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="B31" s="2">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2" t="s">
-        <v>56</v>
+        <v>123</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>57</v>
+        <v>124</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>70</v>
+        <v>7</v>
       </c>
       <c r="B32" s="2">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>125</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2" t="s">
-        <v>156</v>
+        <v>123</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="B33" s="2">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>170</v>
+        <v>133</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2" t="s">
-        <v>171</v>
+        <v>134</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B34" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>262</v>
+        <v>244</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="F34" s="2"/>
+        <v>150</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>216</v>
+      </c>
       <c r="G34" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>155</v>
+        <v>221</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B35" s="2">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="B36" s="2">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>67</v>
+        <v>252</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2" t="s">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="B37" s="2">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>72</v>
+        <v>252</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2" t="s">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>74</v>
+        <v>19</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B38" s="2">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>140</v>
+        <v>252</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>48</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2" t="s">
-        <v>141</v>
+        <v>49</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>142</v>
+        <v>50</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" s="2">
+        <v>63</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B39" s="2">
-        <v>1</v>
-      </c>
-      <c r="C39" s="3" t="s">
+      <c r="B40" s="2">
+        <v>3</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I39" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B40" s="2">
-        <v>72</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="D40" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>121</v>
+        <v>252</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2" t="s">
-        <v>117</v>
+        <v>55</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B41" s="2">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>75</v>
+        <v>252</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2" t="s">
-        <v>76</v>
+        <v>188</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>77</v>
+        <v>189</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="B42" s="2">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>158</v>
+        <v>272</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B43" s="2">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>112</v>
+        <v>168</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2" t="s">
-        <v>113</v>
+        <v>169</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>114</v>
+        <v>170</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B44" s="2">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>81</v>
+        <v>152</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>82</v>
+        <v>153</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>83</v>
+        <v>154</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="165" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B45" s="2">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>41</v>
+        <v>271</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F45" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>211</v>
+      </c>
       <c r="G45" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>44</v>
+        <v>213</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B46" s="2">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>128</v>
+        <v>254</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="2" t="s">
-        <v>129</v>
+        <v>35</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>130</v>
+        <v>36</v>
       </c>
       <c r="I46" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B47" s="2">
+        <v>12</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B48" s="2">
+        <v>4</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B47" s="2">
-        <v>25</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="I47" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
+      <c r="G48" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B49" s="2">
+        <v>48</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B50" s="2">
+        <v>60</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B48" s="2">
-        <v>53</v>
-      </c>
-      <c r="C48" s="3" t="s">
+      <c r="D50" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E50" s="10" t="s">
         <v>71</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="I48" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B49" s="2">
-        <v>27</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="I49" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B50" s="2">
-        <v>65</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="225" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="B51" s="2">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>258</v>
+        <v>118</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="F51" s="2"/>
+        <v>119</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>211</v>
+      </c>
       <c r="G51" s="2" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>103</v>
+        <v>214</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="285" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B52" s="2">
         <v>15</v>
       </c>
-      <c r="B52" s="2">
-        <v>24</v>
-      </c>
       <c r="C52" s="3" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>189</v>
+        <v>268</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>190</v>
+        <v>269</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="I52" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>270</v>
+      </c>
+      <c r="I52" s="4"/>
+    </row>
+    <row r="53" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="B53" s="2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>78</v>
+        <v>265</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>139</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" s="13" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A54" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B54" s="10">
+        <v>74</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>265</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F54" s="10"/>
+      <c r="G54" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H54" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="H53" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I53" s="4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B54" s="2">
-        <v>61</v>
-      </c>
-      <c r="C54" s="3" t="s">
+      <c r="I54" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B55" s="2">
         <v>11</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="A55" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B55" s="2">
-        <v>52</v>
-      </c>
       <c r="C55" s="3" t="s">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>143</v>
+        <v>29</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>144</v>
+        <v>206</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B56" s="2">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>255</v>
+        <v>114</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>148</v>
+        <v>115</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>149</v>
+        <v>116</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>227</v>
+        <v>117</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B57" s="2">
+        <v>72</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B57" s="2">
-        <v>39</v>
-      </c>
-      <c r="C57" s="3" t="s">
+      <c r="B58" s="2">
+        <v>34</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="F57" s="2"/>
-      <c r="G57" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="H57" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="I57" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" ht="180" x14ac:dyDescent="0.25">
-      <c r="A58" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B58" s="2"/>
-      <c r="C58" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="D58" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>237</v>
+        <v>243</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2" t="s">
-        <v>242</v>
+        <v>75</v>
       </c>
       <c r="H58" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="2">
+        <v>43</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="I58" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="210" x14ac:dyDescent="0.25">
-      <c r="A59" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B59" s="2"/>
-      <c r="C59" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="E59" s="2" t="s">
-        <v>235</v>
+        <v>157</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2" t="s">
-        <v>240</v>
+        <v>158</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>241</v>
+        <v>159</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B60" s="2">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D60" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B61" s="2">
+        <v>44</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B62" s="2">
+        <v>36</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B63" s="2">
+        <v>76</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="E60" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="I60" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="A61" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B61" s="2">
-        <v>32</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="G61" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="I61" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B62" s="2">
-        <v>21</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="G62" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="I62" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" ht="165" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B63" s="2">
-        <v>17</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>264</v>
-      </c>
       <c r="E63" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F63" s="5" t="s">
-        <v>218</v>
+        <v>104</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>222</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="H63" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="I63" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="I63" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B64" s="2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C64" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B65" s="2">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>224</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="F65" s="2"/>
       <c r="G65" s="2" t="s">
-        <v>198</v>
+        <v>81</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>230</v>
+        <v>82</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="225" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B66" s="2">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>119</v>
+        <v>40</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>213</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="F66" s="2"/>
       <c r="G66" s="2" t="s">
-        <v>117</v>
+        <v>42</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>216</v>
+        <v>43</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B67" s="2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D67" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I67" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B68" s="2">
+        <v>31</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="E67" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="G67" s="2" t="s">
+      <c r="E68" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H68" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="H67" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="I67" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="105" x14ac:dyDescent="0.25">
-      <c r="A68" s="2" t="s">
+      <c r="I68" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B69" s="2">
         <v>20</v>
       </c>
-      <c r="B68" s="2">
-        <v>44</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="F68" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="G68" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="H68" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="I68" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" ht="105" x14ac:dyDescent="0.25">
-      <c r="A69" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B69" s="2">
-        <v>36</v>
-      </c>
       <c r="C69" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>224</v>
-      </c>
+        <v>246</v>
+      </c>
+      <c r="E69" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="F69" s="2"/>
       <c r="G69" s="2" t="s">
-        <v>169</v>
+        <v>128</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>229</v>
+        <v>129</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="210" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B70" s="2">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>104</v>
+        <v>16</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>224</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="F70" s="2"/>
       <c r="G70" s="2" t="s">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>225</v>
+        <v>277</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="B71" s="2">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>217</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="F71" s="2"/>
       <c r="G71" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I71" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B72" s="2">
+        <v>27</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B73" s="2">
         <v>65</v>
       </c>
-      <c r="H71" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="I71" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="A72" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B72" s="2">
-        <v>15</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="H72" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="I72" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" ht="120" x14ac:dyDescent="0.25">
-      <c r="A73" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B73" s="2">
-        <v>31</v>
-      </c>
       <c r="C73" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>269</v>
+        <v>256</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>217</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="F73" s="2"/>
       <c r="G73" s="2" t="s">
-        <v>211</v>
+        <v>61</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>210</v>
+        <v>62</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" ht="285" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="B74" s="2">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>270</v>
+        <v>100</v>
       </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2" t="s">
-        <v>271</v>
+        <v>101</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>272</v>
+        <v>102</v>
+      </c>
+      <c r="I74" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I73" xr:uid="{5281F1CC-6024-4EAE-8684-9E904383911E}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I73">
-      <sortCondition ref="I1:I73"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:I74" xr:uid="{5281F1CC-6024-4EAE-8684-9E904383911E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>